<commit_message>
MOD Modificado docker con /public como principal y alias en conf para frontend y etc. así como mods a rutas
</commit_message>
<xml_diff>
--- a/uploads/productes.xlsx
+++ b/uploads/productes.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="22">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -440,8 +440,97 @@
         <v>20</v>
       </c>
     </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F8" s="5"/>
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E10" s="5"/>

</xml_diff>

<commit_message>
ADD productos repetidos en json
</commit_message>
<xml_diff>
--- a/uploads/productes.xlsx
+++ b/uploads/productes.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="27">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -86,6 +86,21 @@
   </si>
   <si>
     <t xml:space="preserve">A004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asdsad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asdasd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.20</t>
   </si>
 </sst>
 </file>
@@ -174,7 +189,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -196,6 +211,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -322,7 +341,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -533,8 +552,50 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
+      <c r="A10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="0" t="n">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
MOD Prods y comentarios añadido
</commit_message>
<xml_diff>
--- a/uploads/productes.xlsx
+++ b/uploads/productes.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="52">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -85,19 +85,94 @@
     <t xml:space="preserve">img/raton</t>
   </si>
   <si>
-    <t xml:space="preserve">A004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">asdsad</t>
+    <t xml:space="preserve">G001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baldur's Gate III</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RPG de fantasía épica, ganador de múltiples premios.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">img/baldurs_gate.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">69.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celeste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plataformas de precisión aclamado por la crítica.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">img/celeste.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hogwarts Legacy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RPG de acción ambientado en el mundo mágico de Harry Potter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">img/hogwarts_legacy.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">59.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Windows 11 OEM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Licencia original para instalación de sistema operativo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">img/windows11.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">119.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuphead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run and Gun clásico con estilo de animación de los años 30.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">img/cuphead.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Borderlands 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuevo título de la saga shooter looter (Pre-order).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">img/borderlands4.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A005</t>
   </si>
   <si>
     <t xml:space="preserve">asdasd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50.20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A005</t>
   </si>
   <si>
     <t xml:space="preserve">20.20</t>
@@ -189,7 +264,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -211,10 +286,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -444,19 +515,19 @@
         <v>21</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -464,22 +535,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -487,22 +558,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -510,22 +581,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -533,67 +604,67 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>20</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G11" s="0" t="n">
+      <c r="B11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G11" s="3" t="n">
         <v>20</v>
       </c>
     </row>

</xml_diff>